<commit_message>
cfo.ai numbers: workbook and docs at the measured $0.0085 per audit
The live cfo.ai model already held the measured cost; the repo still showed
the $0.048 estimate. Rebuild results/business_model.xlsx with Assumptions!B5
= $0.0085 (mean neatlogs cost of the three M2 after-audits) and update the
CFO_AI results table, STATUS and spec notes. verify_model.py: 763 formulas,
0 errors, all checks pass, and every figure matches live cfo.ai to the cent
(Base month-12 cash $2,193; Growth needs $47,346).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/business_model.xlsx
+++ b/results/business_model.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="10">
-    <numFmt numFmtId="164" formatCode="$0.000"/>
+    <numFmt numFmtId="164" formatCode="$0.0000"/>
     <numFmt numFmtId="165" formatCode="$#,##0.00;($#,##0.00);&quot;-&quot;"/>
     <numFmt numFmtId="166" formatCode="#,##0;(#,##0);&quot;-&quot;"/>
     <numFmt numFmtId="167" formatCode="0.0%;(0.0%);&quot;-&quot;"/>
@@ -113,12 +113,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
+        <fgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9E1F2"/>
+        <fgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -157,7 +157,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -174,16 +174,16 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="8" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="8" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="8" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="8" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="8" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="8" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="8" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="8" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="169" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -193,8 +193,8 @@
     <xf numFmtId="170" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="171" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="6" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="172" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -583,7 +583,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Two scenarios over 12 months, priced per audit. Change inputs on the Assumptions sheet; everything here recalculates. LLM cost per audit is an ESTIMATE (Assumptions!B5) until M2 measures it.</t>
+          <t>Two scenarios over 12 months, priced per audit. Change inputs on the Assumptions sheet; everything here recalculates. LLM cost per audit is MEASURED (Assumptions!B5).</t>
         </is>
       </c>
     </row>
@@ -612,7 +612,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>LLM cost per audit (ESTIMATE, Assumptions!B5)</t>
+          <t>LLM cost per audit (MEASURED, Assumptions!B5)</t>
         </is>
       </c>
       <c r="B5" s="5">
@@ -1026,14 +1026,14 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>- LLM cost per audit is a bottom-up ESTIMATE from the code (Cost_Estimate sheet), at DeepSeek peak prices. It is replaced with the measured figure after M2.</t>
+          <t>- LLM cost per audit is MEASURED: the mean neatlogs cost of the three M2 after-audits. The pre-M2 bottom-up estimate (Cost_Estimate sheet) was about 5.6x higher.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>- Variable cost is a few cents an audit, so margins are set by price and card fees; the plan is decided by users, churn, CAC and team cost (owner estimates, yellow on Assumptions).</t>
+          <t>- Variable cost is under a cent an audit, so margins are set by price and card fees; the plan is decided by users, churn, CAC and team cost (owner estimates, yellow on Assumptions).</t>
         </is>
       </c>
     </row>
@@ -1089,15 +1089,15 @@
     <row r="5" ht="64" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>LLM cost per audit (USD): ESTIMATE</t>
+          <t>LLM cost per audit (USD): MEASURED</t>
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>0.048</v>
+        <v>0.008500000000000001</v>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>ESTIMATE</t>
+          <t>MEASURED</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
@@ -1107,7 +1107,7 @@
       </c>
       <c r="E5" s="17" t="inlineStr">
         <is>
-          <t>THE single cost variable; both scenarios and every sheet use it. Estimate, not measured: built bottom-up on the Cost_Estimate sheet (0.0476, rounded) from calls per audit, prompt sizes in src/auditor/agents.py and DeepSeek prices in src/llm.py (peak, cache-miss: an upper bound). After M2, type the measured mean cost per audit here: section '9. Cost and trace' of each demo report (cost.usd in state.json), or the neatlogs traces.</t>
+          <t>THE single cost variable; both scenarios and every sheet use it. Measured: mean neatlogs cost of the three M2 after-audits ($0.0114, $0.0056, $0.0085). The wrapper's cost.usd in state.json uses DeepSeek peak cache-miss prices, an upper bound (mean $0.0351). The pre-M2 bottom-up estimate was $0.0476 (Cost_Estimate sheet).</t>
         </is>
       </c>
     </row>
@@ -1615,7 +1615,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>How Assumptions!B5 was estimated before any real audit ran (AUDITOR_SPEC sections 8 and 13). Replace Assumptions!B5 with the measured figure after M2; this sheet then documents the estimate.</t>
+          <t>How Assumptions!B5 was estimated before any real audit ran (AUDITOR_SPEC sections 8 and 13). Assumptions!B5 now holds the measured figure; this sheet documents the estimate.</t>
         </is>
       </c>
     </row>
@@ -2184,7 +2184,7 @@
       </c>
       <c r="D26" s="17" t="inlineStr">
         <is>
-          <t>The bottom-up estimate. Rounded, it is the typed value of Assumptions!B5.</t>
+          <t>The bottom-up estimate, the typed value of Assumptions!B5 until M2.</t>
         </is>
       </c>
     </row>
@@ -2205,7 +2205,7 @@
       </c>
       <c r="D27" s="17" t="inlineStr">
         <is>
-          <t>Green link. Holds this estimate until M2, then the measured figure.</t>
+          <t>Green link. The measured figure (neatlogs, three M2 after-audits).</t>
         </is>
       </c>
     </row>
@@ -2226,7 +2226,7 @@
       </c>
       <c r="D28" s="17" t="inlineStr">
         <is>
-          <t>Under $0.0005 while B5 is still the estimate (rounding).</t>
+          <t>Negative: real audits cost less than the estimate.</t>
         </is>
       </c>
     </row>
@@ -2450,7 +2450,7 @@
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>To replace the estimate: type the mean measured cost per audit of the demo audits into Assumptions!B5. Source: section '9. Cost and trace' of each report.md (or cost.usd in state.json), cross-checked in neatlogs.</t>
+          <t>Replaced: Assumptions!B5 holds the mean measured cost per audit of the three M2 after-audits in neatlogs. The wrapper's cost.usd in each state.json uses peak cache-miss prices, so it is an upper bound (mean $0.0351).</t>
         </is>
       </c>
     </row>
@@ -2519,7 +2519,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>All values in $ unless the unit column says otherwise. Inputs live on the Assumptions sheet, column B; LLM cost per audit is the single cell Assumptions!B5 (ESTIMATE).</t>
+          <t>All values in $ unless the unit column says otherwise. Inputs live on the Assumptions sheet, column B; LLM cost per audit is the single cell Assumptions!B5 (MEASURED).</t>
         </is>
       </c>
     </row>
@@ -4190,7 +4190,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>All values in $ unless the unit column says otherwise. Inputs live on the Assumptions sheet, column C; LLM cost per audit is the single cell Assumptions!B5 (ESTIMATE).</t>
+          <t>All values in $ unless the unit column says otherwise. Inputs live on the Assumptions sheet, column C; LLM cost per audit is the single cell Assumptions!B5 (MEASURED).</t>
         </is>
       </c>
     </row>
@@ -5851,7 +5851,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>LLM cost per audit is Assumptions!B5 (ESTIMATE until M2 measures it).</t>
+          <t>LLM cost per audit is Assumptions!B5 (MEASURED in neatlogs).</t>
         </is>
       </c>
     </row>
@@ -5927,7 +5927,7 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>LLM cost per audit (ESTIMATE)</t>
+          <t>LLM cost per audit (MEASURED)</t>
         </is>
       </c>
       <c r="B7" s="5">

</xml_diff>